<commit_message>
Reescreve textos dos lugares de Sorocaba no tom de voz da marca
Descrições, frases de destaque, dicas, motivos e SEO passam a ter
redação própria, seguindo o tom de voz do design system, sem trechos
próximos das fontes. Fatos sem confirmação foram retirados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MTEVwmA4cVt69NRY1UfnTL
</commit_message>
<xml_diff>
--- a/dados/lugares-sorocaba.xlsx
+++ b/dados/lugares-sorocaba.xlsx
@@ -254,7 +254,7 @@
     </comment>
     <comment ref="H7" authorId="0" shapeId="0">
       <text>
-        <t>Fontes divergem: 2 ou 3 lagos. Texto diz 'lagos' para não errar.</t>
+        <t>Fontes divergem: 2 ou 3 lagos. Texto não cita o número.</t>
       </text>
     </comment>
     <comment ref="W7" authorId="0" shapeId="0">
@@ -264,7 +264,7 @@
     </comment>
     <comment ref="H8" authorId="0" shapeId="0">
       <text>
-        <t>Área: 162 mil m² na maioria das fontes; algumas citam 167 mil m².</t>
+        <t>Área: 162 mil m² na maioria das fontes; algumas citam 167 mil m². Não citado no texto.</t>
       </text>
     </comment>
     <comment ref="W8" authorId="0" shapeId="0">
@@ -575,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -608,109 +608,116 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
+          <t>Textos editoriais (frase de destaque, descrição, dica, motivos, frase da foto, SEO) são autorais, no tom de voz do design system ('amigo que mora na cidade há 10 anos'). Os fatos citados vêm das fontes; a redação não copia nenhuma delas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
           <t>Sugerido pela curadoria a partir do que foi encontrado. Revisar antes de publicar.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-    </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Abas</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Lugares: uma linha por lugar, uma coluna por campo do editor de Lugares do admin. A 2ª linha traz a chave do campo no sistema.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Fontes: links consultados por lugar.</t>
+          <t>Lugares: uma linha por lugar, uma coluna por campo do editor de Lugares do admin. A 2ª linha traz a chave do campo no sistema.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Referências externas: notas do Google, Tripadvisor etc. (apenas consulta).</t>
+          <t>Fontes: links consultados por lugar.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>Referências externas: notas do Google, Tripadvisor etc. (apenas consulta).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>Pendências: o que validar ou cadastrar antes de publicar.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Valores aceitos</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Tipo: Restaurantes, Bares, Parques, Shows e baladas, Eventos</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Faixa de preço: 0 = Grátis · 1 = R$ 30–60 · 2 = R$ 60–120 · 3 = R$ 150–300</t>
+          <t>Tipo: Restaurantes, Bares, Parques, Shows e baladas, Eventos</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Momento: Jantar, Almoço, Happy hour, Brunch, Noite, Experiência cultural</t>
+          <t>Faixa de preço: 0 = Grátis · 1 = R$ 30–60 · 2 = R$ 60–120 · 3 = R$ 150–300</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Ambiente: Ambiente interno, Ambiente externo</t>
+          <t>Momento: Jantar, Almoço, Happy hour, Brunch, Noite, Experiência cultural</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Vibes (ids): dates, impress, turist, relax, eco, crianca</t>
+          <t>Ambiente: Ambiente interno, Ambiente externo</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Ícones dos motivos: eye, star, heart, users, music, leaf, sun, coins, clock, sparkle, image, camera, wine, smile, pin</t>
+          <t>Vibes (ids): dates, impress, turist, relax, eco, crianca</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Destaques do topo: Vista linda, Boa música, Para ir com amigos, Experiência única, Boa luz, Sem pressa, Para ir com crianças, Programa a dois</t>
+          <t>Ícones dos motivos: eye, star, heart, users, music, leaf, sun, coins, clock, sparkle, image, camera, wine, smile, pin</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Destaques do topo: Vista linda, Boa música, Para ir com amigos, Experiência única, Boa luz, Sem pressa, Para ir com crianças, Programa a dois</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Células com triângulo vermelho têm comentário (conflito entre fontes ou observação).</t>
         </is>
@@ -1214,7 +1221,7 @@
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>Growleria na Vila Santana com 6 torneiras de chope artesanal que giram sempre, além de rótulos nacionais e importados. Dá pra tomar ali mesmo ou encher o growler (vidro, porcelana ou growler bag) e levar pra casa. Clima de bar de bairro, sem frescura.</t>
+          <t>Aquele lugar pra passar depois do trampo, encher o growler e levar cerveja boa pra casa. São 6 torneiras de chope artesanal que trocam o tempo todo, então cada visita tem novidade. Bateu vontade? Encosta no balcão e toma ali mesmo. Bar de bairro na Vila Santana, sem frescura nenhuma.</t>
         </is>
       </c>
       <c r="I3" s="8" t="inlineStr">
@@ -1237,9 +1244,9 @@
           <t>wine | 6 torneiras com rótulos que mudam sempre</t>
         </is>
       </c>
-      <c r="M3" s="8" t="inlineStr">
-        <is>
-          <t>coins | Encher o growler sai mais em conta que chope na mesa</t>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>coins | Chope fresco pra levar no vidro, na porcelana ou na bag</t>
         </is>
       </c>
       <c r="N3" s="9" t="inlineStr">
@@ -1398,7 +1405,7 @@
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t>Pub tradicional no Centro com 12 torneiras de chope artesanal: IPA, APA, Pilsen, Weizen e convidadas que mudam sempre. A cozinha segura bem a onda: hambúrguer no brioche, defumados, charcutaria e porções. Espaço aconchegante, com som ao vivo em algumas noites e almoço aos sábados.</t>
+          <t>Pub de verdade no meio do Centro, com 12 torneiras de chope artesanal que vão mudando de estilo. E a cozinha não é coadjuvante: tem hambúrguer no brioche, defumados e até charcutaria. Rola som ao vivo em algumas noites e, no sábado, abre pro almoço. Daqueles lugares em que você chega pra um chope e sai horas depois.</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
@@ -1423,7 +1430,7 @@
       </c>
       <c r="M4" s="8" t="inlineStr">
         <is>
-          <t>star | Hambúrguer e defumados acima da média de bar</t>
+          <t>star | Cozinha que vai muito além da porção de fritas</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
@@ -1586,12 +1593,12 @@
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>Bar y parrilla do churrasqueiro Felipe Botti, com raízes nos churrascos descontraídos entre amigos. Cortes na brasa no ponto, parrillada mista, empanadas e boa carta pra acompanhar. Ambiente moderno, entre o sofisticado e o alternativo, com serviço rápido e atencioso.</t>
+          <t>Sabe aquele churrasco de amigo que ninguém quer que acabe? O Carneada levou essa ideia pra parrilla, com sotaque argentino. O churrasqueiro Felipe Botti comanda a brasa, a parrillada chega pra dividir na mesa e as empanadas seguram a fome enquanto a carne fica pronta. Fica no Centro, num espaço moderno que não pesa no clima.</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>Vá em turma e divida a parrillada mista. Abra com empanadas enquanto a brasa trabalha. No almoço de semana a casa fica mais tranquila.</t>
+          <t>Vá em turma e divida a parrillada mista. Abra com empanadas enquanto a brasa trabalha. Domingo fecha às 16h: não deixe pra ir tarde.</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
@@ -1728,7 +1735,7 @@
       </c>
       <c r="AN5" s="8" t="inlineStr">
         <is>
-          <t>Parrilla do churrasqueiro Felipe Botti: cortes na brasa, parrillada mista e empanadas num ambiente moderno no Centro de Sorocaba.</t>
+          <t>Churrasco de amigo com sotaque argentino: parrillada pra dividir, empanadas e brasa comandada por Felipe Botti, no Centro de Sorocaba.</t>
         </is>
       </c>
     </row>
@@ -1768,9 +1775,9 @@
           <t>Brisket, costela e pulled pork defumados por horas, no melhor estilo Texas.</t>
         </is>
       </c>
-      <c r="H6" s="9" t="inlineStr">
-        <is>
-          <t>Autêntico churrasco americano no Jardim Paulistano: brisket, ribs e pulled pork defumados lentamente no pit smoker com lenha de árvores frutíferas. Vem com molhos da casa, coleslaw e cornbread. No fim de semana abre cedo com café da manhã americano: bacon, ovos, linguiça e panquecas.</t>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Churrasco americano raiz em Sorocaba, coisa que não se acha em qualquer esquina. A carne passa horas no defumador com lenha de árvore frutífera até ficar macia e com aquele gosto de fumaça. Vem com molho da casa, coleslaw e cornbread. E no fim de semana tem café da manhã americano, com panqueca, bacon e ovo.</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr">
@@ -1800,7 +1807,7 @@
       </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
-          <t>sparkle | Barbecue texano de verdade, raro na cidade</t>
+          <t>sparkle | Barbecue americano de verdade, raro na cidade</t>
         </is>
       </c>
       <c r="O6" s="8" t="inlineStr">
@@ -1949,12 +1956,12 @@
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>Lagos, trilha curtinha e bichos de perto, de graça, no Jardim Europa.</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
-          <t>Parque natural de 20 mil m² inaugurado em 1990, com lagos cercados de árvores frutíferas, trilha em volta da água e bichos como cágados, garças e pica-paus. Tem aquário, jardim sensorial, biblioteca, playground, quiosques e mesas de piquenique. Reabriu depois do desassoreamento do lago.</t>
+          <t>Garça, cágado e trilha em volta do lago, de graça, no meio do Jardim Europa.</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Um respiro verde no Jardim Europa, onde dá pra ver garça, cágado e pica-pau sem sair da cidade. A trilha contorna os lagos sem pressa, a criançada se diverte entre aquário, playground e jardim sensorial, e as mesas de piquenique esperam o lanche que você trouxer. E a entrada é de graça.</t>
         </is>
       </c>
       <c r="I7" s="8" t="inlineStr">
@@ -1974,7 +1981,7 @@
       </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
-          <t>heart | Garças, cágados e pica-paus de pertinho</t>
+          <t>heart | Garça, cágado e pica-pau de pertinho</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
@@ -2100,7 +2107,7 @@
       </c>
       <c r="AN7" s="8" t="inlineStr">
         <is>
-          <t>Lagos, trilha, aquário e bichos de perto no Jardim Europa. Entrada gratuita, de terça a domingo, das 8h às 17h.</t>
+          <t>Garça, cágado, trilha em volta do lago e aquário pra criançada no Jardim Europa. De graça, de terça a domingo.</t>
         </is>
       </c>
     </row>
@@ -2137,12 +2144,12 @@
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>162 mil m² de lagos, ciclovia e pista de skate, aberto 24 horas e de graça.</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr">
-        <is>
-          <t>Um dos maiores parques de Sorocaba, inaugurado em 2008 numa antiga área de enchentes ao lado do rio Sorocaba. São 162 mil m² com três lagos, fonte, deck de madeira, pista de caminhada, ciclovia, pistas de skate, playground, quadras e anfiteatro. Recebe shows e eventos da cidade.</t>
+          <t>Lago, ciclovia, skate e gramado pra perder a hora. Aberto 24 horas e de graça.</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>É pra cá que Sorocaba vem quando quer se mexer. O parque nasceu numa antiga área de enchente na beira do rio e virou um quintal gigante, com lagos, deck de madeira, ciclovia, pista de skate e muito gramado. Fica aberto dia e noite, todo dia, sem pagar nada. Quando tem show ou evento grande na cidade, é bem capaz de ser aqui.</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
@@ -2162,12 +2169,12 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>leaf | Três lagos, fonte e deck de madeira</t>
+          <t>sun | Fim de tarde no deck, de frente pro lago</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>clock | Aberto 24 horas, todos os dias</t>
+          <t>clock | Aberto dia e noite, todo dia</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
@@ -2280,7 +2287,7 @@
       </c>
       <c r="AN8" s="8" t="inlineStr">
         <is>
-          <t>162 mil m² à beira do rio Sorocaba com lagos, ciclovia, pistas de skate, playground e anfiteatro. Aberto 24 horas e de graça.</t>
+          <t>Lago, ciclovia, skate e gramado à beira do rio Sorocaba. Aberto 24 horas, todo dia, e de graça. Programa certo pro fim de tarde.</t>
         </is>
       </c>
     </row>
@@ -2305,9 +2312,9 @@
           <t>Drink Me Speakeasy Bar</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>Speakeasy de alta coquetelaria</t>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Speakeasy de drinques autorais</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
@@ -2317,17 +2324,17 @@
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>O primeiro speakeasy de Sorocaba: drinques de técnica apurada e luz baixa.</t>
-        </is>
-      </c>
-      <c r="H9" s="9" t="inlineStr">
-        <is>
-          <t>Primeiro e único bar inspirado no conceito speakeasy em Sorocaba, focado em alta coquetelaria. Clássicos e autorais executados com precisão, num ambiente intimista ao som de jazz e blues. Pra comer, schiacciatas artesanais feitas na casa. Funciona só com reserva.</t>
+          <t>O único speakeasy de Sorocaba: luz baixa, jazz e coquetel feito com capricho.</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>Clima de bar clandestino dos anos 20, só que em Sorocaba: o Drink Me é o único speakeasy da cidade. Luz baixa, jazz e blues no som e gente que leva coquetel a sério, dos clássicos aos autorais da casa. Pra beliscar, schiacciata feita ali mesmo. Só entra com reserva, então se programe.</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>Reserve antes: a casa atende exclusivamente com reserva. Peça o Garden Mule, queridinho de quem já foi, e divida uma schiacciata.</t>
+          <t>Sem reserva não rola, então garanta a sua antes. Peça o Garden Mule e pergunte a história dele. Divida uma schiacciata.</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
@@ -2347,7 +2354,7 @@
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>wine | Drinques autorais de alta coquetelaria</t>
+          <t>wine | Coquetel levado a sério, do clássico ao autoral</t>
         </is>
       </c>
       <c r="N9" s="9" t="inlineStr">
@@ -2463,12 +2470,12 @@
       </c>
       <c r="AM9" s="8" t="inlineStr">
         <is>
-          <t>Drink Me · Speakeasy e alta coquetelaria em Sorocaba</t>
+          <t>Drink Me · O speakeasy de Sorocaba</t>
         </is>
       </c>
       <c r="AN9" s="8" t="inlineStr">
         <is>
-          <t>O primeiro speakeasy de Sorocaba: drinques clássicos e autorais, jazz, schiacciatas da casa e atendimento só com reserva.</t>
+          <t>O único speakeasy de Sorocaba: luz baixa, jazz, coquetel caprichado e schiacciata da casa. Só com reserva, então se programe.</t>
         </is>
       </c>
     </row>

</xml_diff>